<commit_message>
Publish Bratislava_2011_WCH, Deodoro_2016_OG, LaSeu_2016_WC
</commit_message>
<xml_diff>
--- a/events/Bratislava_2011_WCH/Bratislava_2011_WCH_start.xlsx
+++ b/events/Bratislava_2011_WCH/Bratislava_2011_WCH_start.xlsx
@@ -31928,7 +31928,7 @@
       </c>
       <c r="I541" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>LBN</t>
         </is>
       </c>
       <c r="J541" t="n">
@@ -37283,7 +37283,7 @@
       </c>
       <c r="I636" t="inlineStr">
         <is>
-          <t>LIB</t>
+          <t>LBN</t>
         </is>
       </c>
       <c r="J636" t="n">

</xml_diff>

<commit_message>
Publish LaSeu_2015_WC, Pau_2016_WC, Bratislava_2011_WCH, Deodoro_2016_OG
</commit_message>
<xml_diff>
--- a/events/Bratislava_2011_WCH/Bratislava_2011_WCH_start.xlsx
+++ b/events/Bratislava_2011_WCH/Bratislava_2011_WCH_start.xlsx
@@ -31942,6 +31942,11 @@
           <t>MERJAN Richard</t>
         </is>
       </c>
+      <c r="X541" t="inlineStr">
+        <is>
+          <t>45918</t>
+        </is>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -37295,6 +37300,11 @@
       <c r="R636" t="inlineStr">
         <is>
           <t>MERJAN Richard</t>
+        </is>
+      </c>
+      <c r="X636" t="inlineStr">
+        <is>
+          <t>45918</t>
         </is>
       </c>
     </row>

</xml_diff>